<commit_message>
Tratamento para registro do kardex, desdobramento e grupamento e sobra
</commit_message>
<xml_diff>
--- a/template kardex.xlsx
+++ b/template kardex.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="22">
   <si>
     <t>Data lançamento</t>
   </si>
@@ -64,6 +64,24 @@
   </si>
   <si>
     <t>CPTS11</t>
+  </si>
+  <si>
+    <t>grupamento</t>
+  </si>
+  <si>
+    <t>qtd_entrada será menor que 0</t>
+  </si>
+  <si>
+    <t>,</t>
+  </si>
+  <si>
+    <t>Então</t>
+  </si>
+  <si>
+    <t>valor movimento = saldo vlr final * -1</t>
+  </si>
+  <si>
+    <t>qtd_entrada resulta em fração</t>
   </si>
 </sst>
 </file>
@@ -72,7 +90,7 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="2">
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
-    <numFmt numFmtId="167" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
+    <numFmt numFmtId="164" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -111,12 +129,14 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="43" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -419,7 +439,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:M6"/>
+  <dimension ref="B2:Q13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="14.7109375" bestFit="1" customWidth="1"/>
@@ -433,7 +453,7 @@
     <col min="13" max="13" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B2" t="s">
         <v>14</v>
       </c>
@@ -471,7 +491,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B3">
         <v>1</v>
       </c>
@@ -491,23 +511,32 @@
         <v>15</v>
       </c>
       <c r="I3" s="2">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="J3">
         <v>100</v>
       </c>
       <c r="K3">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="L3">
         <v>100</v>
       </c>
       <c r="M3" s="4">
         <f>L3/K3</f>
-        <v>100</v>
-      </c>
+        <v>8.3333333333333339</v>
+      </c>
+      <c r="O3" s="6">
+        <f>-M3*(H4-I4*10)</f>
+        <v>-16.666666666666668</v>
+      </c>
+      <c r="P3" s="6">
+        <f>M3*I4*10</f>
+        <v>83.333333333333343</v>
+      </c>
+      <c r="Q3" s="6"/>
     </row>
-    <row r="4" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B4">
         <v>2</v>
       </c>
@@ -518,35 +547,38 @@
         <v>46022</v>
       </c>
       <c r="E4" t="s">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
         <v>15</v>
       </c>
       <c r="H4" s="2">
+        <v>12</v>
+      </c>
+      <c r="I4" s="5">
         <v>1</v>
       </c>
-      <c r="I4" s="2">
-        <v>10</v>
-      </c>
       <c r="J4">
-        <f>L3</f>
-        <v>100</v>
+        <v>-100</v>
       </c>
       <c r="K4" s="3">
         <f>K3-H4+I4</f>
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="L4">
-        <f>L3</f>
-        <v>100</v>
+        <f>L3+J4</f>
+        <v>0</v>
       </c>
       <c r="M4" s="4">
-        <f>L4/K4</f>
-        <v>10</v>
+        <f>IFERROR(L4/K4,0)</f>
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <f>P3/I4</f>
+        <v>83.333333333333343</v>
       </c>
     </row>
-    <row r="5" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B5">
         <v>3</v>
       </c>
@@ -573,18 +605,18 @@
       </c>
       <c r="K5" s="3">
         <f>K4-H5+I5</f>
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="L5">
         <f>L4+J5</f>
-        <v>322</v>
+        <v>222</v>
       </c>
       <c r="M5" s="4">
-        <f>L5/K5</f>
-        <v>26.833333333333332</v>
+        <f>IFERROR(L5/K5,0)</f>
+        <v>74</v>
       </c>
     </row>
-    <row r="6" spans="2:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="2:17" x14ac:dyDescent="0.25">
       <c r="B6">
         <v>4</v>
       </c>
@@ -611,15 +643,42 @@
       </c>
       <c r="K6" s="3">
         <f>K5-H6+I6</f>
-        <v>30</v>
+        <v>21</v>
       </c>
       <c r="L6">
         <f>L5</f>
-        <v>322</v>
+        <v>222</v>
       </c>
       <c r="M6" s="4">
         <f>L6/K6</f>
-        <v>10.733333333333333</v>
+        <v>10.571428571428571</v>
+      </c>
+    </row>
+    <row r="11" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="J11">
+        <v>1</v>
+      </c>
+      <c r="K11" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="J12" t="s">
+        <v>18</v>
+      </c>
+      <c r="K12" t="s">
+        <v>19</v>
+      </c>
+      <c r="L12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="13" spans="2:17" x14ac:dyDescent="0.25">
+      <c r="J13">
+        <v>2</v>
+      </c>
+      <c r="K13" t="s">
+        <v>21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>